<commit_message>
MACD scan results 2026-10-12
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,19 +462,15 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>FHB</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ANIP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -485,19 +481,15 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BSBR</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>IDXX</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -508,7 +500,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>BSBR</t>
         </is>
       </c>
     </row>
@@ -516,7 +508,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -527,7 +519,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
@@ -535,7 +527,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -546,7 +538,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>CDNS</t>
         </is>
       </c>
     </row>
@@ -554,18 +546,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FELE</t>
+          <t>ENSG</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>CGNX</t>
         </is>
       </c>
     </row>
@@ -573,18 +565,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FUTU</t>
+          <t>ERIC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>CORT</t>
         </is>
       </c>
     </row>
@@ -592,18 +584,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>CSCO</t>
         </is>
       </c>
     </row>
@@ -611,18 +603,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
@@ -630,18 +622,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>FELE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>EXTR</t>
         </is>
       </c>
     </row>
@@ -649,18 +641,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>FUTU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>FFIV</t>
         </is>
       </c>
     </row>
@@ -668,18 +660,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>FLEX</t>
         </is>
       </c>
     </row>
@@ -687,18 +679,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>FTNT</t>
         </is>
       </c>
     </row>
@@ -706,7 +698,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -717,7 +709,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MTSI</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
@@ -725,216 +717,284 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>IBRX</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LNT</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>IDCC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LSTR</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RXT</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ODFL</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ORLY</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>VCTR</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>NTAP</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>NWE</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>JOYY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -945,7 +1005,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -956,7 +1016,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -967,7 +1027,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>NDSN</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -978,7 +1038,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -989,7 +1049,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1000,7 +1060,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1011,7 +1071,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1022,7 +1082,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1033,7 +1093,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>RELL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1044,7 +1104,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>RZLT</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1055,7 +1115,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1066,7 +1126,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1077,7 +1137,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>SKWD</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1088,7 +1148,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1099,7 +1159,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>STGW</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1110,7 +1170,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1121,99 +1181,11 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>PRCH</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>QLYS</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>RELL</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>RZLT</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>SKWD</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>XMTR</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-14
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,14 +462,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>AMZN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>SUPN</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -485,7 +485,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
@@ -498,13 +498,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BSBR</t>
+          <t>CSCO</t>
         </is>
       </c>
     </row>
@@ -512,12 +512,12 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ALLT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -531,12 +531,12 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>ENSG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -550,7 +550,7 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>ERIC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -561,7 +561,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EZPW</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -580,7 +580,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
@@ -588,18 +588,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FELE</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -612,13 +612,13 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
@@ -626,18 +626,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
@@ -645,18 +645,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
@@ -664,18 +664,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>ODFL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
@@ -683,18 +683,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RZLT</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -702,18 +702,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CLMT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>PCVX</t>
         </is>
       </c>
     </row>
@@ -721,18 +721,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
@@ -740,72 +740,76 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CLWT</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SUPN</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -816,7 +820,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -827,7 +831,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -838,7 +842,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -849,7 +853,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -860,7 +864,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -871,7 +875,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -882,7 +886,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -893,7 +897,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -904,7 +908,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -915,7 +919,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -926,7 +930,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -937,7 +941,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -948,7 +952,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -959,7 +963,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -970,7 +974,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -981,7 +985,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -992,7 +996,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1003,7 +1007,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1014,7 +1018,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1025,7 +1029,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1036,7 +1040,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1047,7 +1051,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1058,7 +1062,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1113,22 +1117,11 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-15
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,14 +462,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SUPN</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -498,13 +498,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>CHEF</t>
         </is>
       </c>
     </row>
@@ -517,13 +517,13 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>CLOV</t>
         </is>
       </c>
     </row>
@@ -536,13 +536,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
@@ -555,13 +555,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -574,13 +574,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
@@ -593,13 +593,13 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
@@ -607,18 +607,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FUTU</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
@@ -626,18 +626,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -645,18 +645,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -669,13 +669,13 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>PCVX</t>
         </is>
       </c>
     </row>
@@ -688,13 +688,13 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
@@ -707,13 +707,13 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -721,18 +721,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
@@ -740,37 +740,33 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CLWT</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>SHOP</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
@@ -779,37 +775,29 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>STLD</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -820,7 +808,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -831,7 +819,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>EZPW</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -842,7 +830,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -853,7 +841,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -864,7 +852,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -875,7 +863,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -886,7 +874,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -897,7 +885,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -908,7 +896,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -919,7 +907,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -930,7 +918,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -941,7 +929,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -952,7 +940,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -963,7 +951,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -974,7 +962,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -985,7 +973,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -996,7 +984,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1007,7 +995,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1018,110 +1006,11 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>NSIT</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>OPLN</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-16
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -456,25 +456,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ATAT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -485,26 +485,30 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>CLMT</t>
         </is>
       </c>
     </row>
@@ -512,18 +516,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>CASY</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AFRM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
@@ -531,18 +535,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -550,18 +554,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -574,13 +578,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
@@ -593,13 +597,13 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>MSFT</t>
         </is>
       </c>
     </row>
@@ -607,18 +611,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -626,18 +630,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>ONC</t>
         </is>
       </c>
     </row>
@@ -645,12 +649,12 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -664,18 +668,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
@@ -683,18 +687,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>ODFL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -707,13 +711,13 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>SHOP</t>
         </is>
       </c>
     </row>
@@ -721,18 +725,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CHEF</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>STLD</t>
         </is>
       </c>
     </row>
@@ -740,42 +744,38 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VMRK</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -786,7 +786,7 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -797,7 +797,7 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -808,7 +808,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -819,7 +819,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -830,7 +830,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -841,7 +841,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -852,7 +852,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>ECPG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -863,7 +863,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -874,7 +874,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -885,7 +885,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>EZPW</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -896,7 +896,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -907,7 +907,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -918,7 +918,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -929,7 +929,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -940,7 +940,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -951,7 +951,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -962,7 +962,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -973,7 +973,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -984,7 +984,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -995,7 +995,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1006,11 +1006,154 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MTCH</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SHOO</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-17
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,12 +451,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ATAT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -469,23 +469,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATAT</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
@@ -497,18 +497,18 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>CASY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
@@ -516,18 +516,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>CDZI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -540,13 +540,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
@@ -559,13 +559,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ALLT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
@@ -573,18 +573,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>ESLT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -592,18 +592,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ECPG</t>
         </is>
       </c>
     </row>
@@ -611,18 +611,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -630,18 +630,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -649,18 +649,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
@@ -668,18 +668,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BCPC</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>MTCH</t>
         </is>
       </c>
     </row>
@@ -692,13 +692,13 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -736,7 +736,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -753,7 +753,11 @@
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SHOO</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
@@ -768,7 +772,11 @@
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
@@ -779,7 +787,11 @@
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
@@ -790,7 +802,11 @@
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -819,7 +835,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -830,7 +846,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -841,7 +857,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -852,7 +868,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ECPG</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -863,7 +879,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -874,7 +890,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -885,7 +901,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -896,7 +912,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -907,7 +923,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -918,7 +934,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -929,7 +945,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -940,7 +956,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -951,7 +967,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -962,7 +978,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -973,7 +989,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -984,7 +1000,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -995,7 +1011,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1006,7 +1022,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1017,7 +1033,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1028,132 +1044,11 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>NWSA</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>PLMR</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>SHOO</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-20
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,7 +447,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ATAT</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -458,7 +458,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -477,7 +477,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
@@ -485,7 +485,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -496,7 +496,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -515,7 +515,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
@@ -523,18 +523,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -542,18 +542,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -561,18 +561,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ESLT</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -580,18 +580,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
@@ -599,18 +599,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ECPG</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
@@ -618,18 +618,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -637,18 +637,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BCPC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -656,220 +656,156 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>OSIS</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>SHOO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>OZK</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PECO</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>LAUR</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>PNFP</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>LGND</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>NTES</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>NWSA</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>OPLN</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>POWW</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>SHOO</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -880,7 +816,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -891,7 +827,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -902,7 +838,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -913,7 +849,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -924,7 +860,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -946,7 +882,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -957,7 +893,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -968,7 +904,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -979,7 +915,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -990,7 +926,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1001,7 +937,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1012,7 +948,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1023,7 +959,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1034,7 +970,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1045,7 +981,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1056,7 +992,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1067,7 +1003,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1078,7 +1014,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1089,7 +1025,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1100,7 +1036,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1111,7 +1047,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1122,7 +1058,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1133,7 +1069,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1144,7 +1080,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1155,7 +1091,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1166,7 +1102,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1177,7 +1113,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1188,7 +1124,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1199,7 +1135,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1210,11 +1146,110 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-21
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,7 +447,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -458,7 +458,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
@@ -466,18 +466,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>AFRM</t>
         </is>
       </c>
     </row>
@@ -485,18 +485,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
@@ -504,18 +504,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>CRMD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -534,7 +534,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
@@ -542,18 +542,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -561,18 +561,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
@@ -580,18 +580,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
@@ -599,18 +599,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -629,7 +629,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
@@ -637,18 +637,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>MIDD</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>CORT</t>
         </is>
       </c>
     </row>
@@ -656,156 +656,224 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>BTSG</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>OSIS</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SHOO</t>
+          <t>CYRX</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OZK</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>FANG</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GSAT</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>KDP</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LGND</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>VMRK</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -816,7 +884,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -827,7 +895,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -838,7 +906,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -860,7 +928,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -871,7 +939,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -882,7 +950,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -893,7 +961,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -904,7 +972,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -915,7 +983,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -926,7 +994,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -937,7 +1005,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -948,7 +1016,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -959,7 +1027,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>JOYY</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -970,7 +1038,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -981,7 +1049,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -992,7 +1060,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1003,7 +1071,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1014,7 +1082,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1025,7 +1093,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1036,7 +1104,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1047,7 +1115,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1058,7 +1126,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1069,7 +1137,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1080,7 +1148,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1091,7 +1159,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1102,7 +1170,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>ORIC</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1113,7 +1181,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1124,7 +1192,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1135,7 +1203,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1146,7 +1214,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1157,7 +1225,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1168,7 +1236,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1179,7 +1247,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1190,7 +1258,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1201,7 +1269,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>SEIC</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1212,7 +1280,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>SEZL</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1223,7 +1291,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1234,7 +1302,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>SLN</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1245,11 +1313,55 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-22
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,21 +444,25 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ABNB</t>
         </is>
       </c>
     </row>
@@ -466,18 +470,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
@@ -485,18 +489,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>CARG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -504,18 +508,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CASH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
@@ -534,7 +538,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -553,7 +557,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
@@ -566,13 +570,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -585,13 +589,13 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
@@ -599,18 +603,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
@@ -618,18 +622,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
@@ -637,18 +641,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MIDD</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
@@ -656,18 +660,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
@@ -675,18 +679,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -694,18 +698,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CRON</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EXPE</t>
         </is>
       </c>
     </row>
@@ -713,12 +717,12 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>RYAAY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -732,18 +736,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>TBLA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>FROG</t>
         </is>
       </c>
     </row>
@@ -751,66 +755,54 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>RYAAY</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CYRX</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>DAVE</t>
@@ -819,7 +811,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
@@ -834,7 +826,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>MNST</t>
         </is>
       </c>
     </row>
@@ -843,13 +835,13 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>DCOM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>NTNX</t>
         </is>
       </c>
     </row>
@@ -858,13 +850,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -873,11 +865,15 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PAYO</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
@@ -888,36 +884,48 @@
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -961,7 +969,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -983,7 +991,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -994,7 +1002,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1027,7 +1035,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1038,7 +1046,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1060,7 +1068,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1071,7 +1079,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1082,7 +1090,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1093,7 +1101,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1104,7 +1112,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1115,7 +1123,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1126,7 +1134,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1137,7 +1145,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1203,7 +1211,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1214,7 +1222,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1225,7 +1233,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1236,7 +1244,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1247,7 +1255,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1258,7 +1266,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1269,7 +1277,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1280,7 +1288,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>SEIC</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1291,7 +1299,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>SEZL</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1302,7 +1310,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1313,7 +1321,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>SLN</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1324,7 +1332,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1335,7 +1343,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TNGX</t>
+          <t>STLN</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1346,7 +1354,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>TNGX</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1357,11 +1365,33 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>UTHR</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-23
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,14 +444,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>ANIP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -470,7 +466,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -489,7 +485,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -508,7 +504,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -519,7 +515,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -527,18 +523,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CRMD</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
@@ -546,18 +542,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>BOKF</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>CLOV</t>
         </is>
       </c>
     </row>
@@ -565,18 +561,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>CARG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>CRSR</t>
         </is>
       </c>
     </row>
@@ -584,18 +580,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>CASH</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -603,18 +599,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>CRMD</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -622,18 +618,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
@@ -641,18 +637,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
@@ -660,18 +656,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>IRTC</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>BCPC</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
@@ -679,18 +675,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
@@ -698,18 +694,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>MIDD</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>MTCH</t>
         </is>
       </c>
     </row>
@@ -717,18 +713,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -736,18 +732,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TBLA</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -755,177 +751,161 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>ROST</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>TECH</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TROO</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>KNSA</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VMRK</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CRON</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>MNST</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>NTNX</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>OPLN</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>PAYO</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>RGEN</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>ROST</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>CYRX</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -936,7 +916,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -947,7 +927,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>DCOM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -958,7 +938,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -969,7 +949,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -980,7 +960,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -991,7 +971,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1002,7 +982,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1013,7 +993,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1024,7 +1004,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1035,7 +1015,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1046,7 +1026,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1057,7 +1037,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1068,7 +1048,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1079,7 +1059,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1090,7 +1070,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1101,7 +1081,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1112,7 +1092,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1123,7 +1103,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1134,7 +1114,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1145,7 +1125,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1156,7 +1136,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1167,7 +1147,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1178,7 +1158,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1189,7 +1169,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1200,7 +1180,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1211,7 +1191,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1222,7 +1202,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1233,7 +1213,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1244,7 +1224,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1255,7 +1235,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1266,7 +1246,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1277,7 +1257,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1288,7 +1268,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1299,7 +1279,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1310,7 +1290,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1321,7 +1301,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1332,7 +1312,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1343,7 +1323,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>ORIC</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1354,7 +1334,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>TNGX</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1365,7 +1345,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1376,7 +1356,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1387,11 +1367,187 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>PAYO</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-24
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,7 +444,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LSTR</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>ANIP</t>
@@ -458,7 +462,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
@@ -466,18 +470,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
@@ -485,18 +489,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -504,18 +508,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
@@ -523,18 +527,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>BLBD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CRON</t>
         </is>
       </c>
     </row>
@@ -547,13 +551,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CRSR</t>
         </is>
       </c>
     </row>
@@ -566,13 +570,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>APPN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CRSR</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -591,7 +595,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
@@ -604,13 +608,13 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
@@ -618,7 +622,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -629,7 +633,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -637,7 +641,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -648,7 +652,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -656,7 +660,7 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -667,7 +671,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>EXPE</t>
         </is>
       </c>
     </row>
@@ -675,7 +679,7 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -686,7 +690,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>FOX</t>
         </is>
       </c>
     </row>
@@ -694,7 +698,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MIDD</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -705,7 +709,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>FOXA</t>
         </is>
       </c>
     </row>
@@ -713,7 +717,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -724,7 +728,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>FTNT</t>
         </is>
       </c>
     </row>
@@ -732,18 +736,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CENTA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
@@ -751,18 +755,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -775,13 +779,13 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
@@ -789,222 +793,282 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>TROO</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LLYVK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MTCH</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>OPLN</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ORIC</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PAYO</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1015,7 +1079,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1026,7 +1090,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1037,7 +1101,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1048,7 +1112,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1059,7 +1123,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1070,7 +1134,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1081,7 +1145,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1092,7 +1156,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1103,7 +1167,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1114,7 +1178,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1125,7 +1189,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1136,7 +1200,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1147,7 +1211,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1158,7 +1222,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>NWBI</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1169,7 +1233,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1180,7 +1244,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1191,7 +1255,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1202,7 +1266,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1213,7 +1277,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1224,7 +1288,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1235,7 +1299,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1246,7 +1310,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>QLYS</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1257,7 +1321,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1268,7 +1332,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1279,7 +1343,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1290,7 +1354,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>SFNC</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1301,7 +1365,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1312,7 +1376,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>UTHR</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1323,7 +1387,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1334,220 +1398,11 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>XNCR</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>PAGP</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>PAYO</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>PLMR</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>QLYS</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>REGN</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>ROKU</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>RPRX</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>SIGI</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr"/>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr"/>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>TNGX</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr"/>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr"/>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr"/>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-26
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,31 +446,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ANIP</t>
+          <t>AMBA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LSTR</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>ANIP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -481,7 +485,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ADI</t>
         </is>
       </c>
     </row>
@@ -489,18 +493,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
@@ -519,7 +523,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
@@ -538,7 +542,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -557,7 +561,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CRSR</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -576,7 +580,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -584,7 +588,7 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -595,7 +599,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
@@ -603,18 +607,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRMD</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -622,7 +626,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -633,7 +637,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -641,7 +645,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -660,18 +664,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>FFIV</t>
         </is>
       </c>
     </row>
@@ -679,12 +683,12 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -698,12 +702,12 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>PATK</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -717,12 +721,12 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>RYAAY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>CENTA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -736,75 +740,63 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>OSIS</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>LIVN</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>TPG</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
@@ -813,13 +805,13 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>MNST</t>
         </is>
       </c>
     </row>
@@ -828,13 +820,13 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -849,7 +841,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>NTNX</t>
         </is>
       </c>
     </row>
@@ -864,7 +856,7 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>NWS</t>
         </is>
       </c>
     </row>
@@ -879,7 +871,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>NWSA</t>
         </is>
       </c>
     </row>
@@ -894,7 +886,7 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -909,7 +901,7 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
@@ -924,7 +916,7 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
@@ -933,13 +925,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -948,13 +940,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>ROKU</t>
         </is>
       </c>
     </row>
@@ -963,13 +955,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
@@ -978,13 +970,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PAYO</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
@@ -993,13 +985,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>SRZN</t>
         </is>
       </c>
     </row>
@@ -1008,13 +1000,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
@@ -1023,52 +1015,40 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>FFBC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>FITB</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1079,7 +1059,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1090,7 +1070,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1101,7 +1081,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>FULT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1112,7 +1092,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1123,7 +1103,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1134,7 +1114,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1145,7 +1125,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1156,7 +1136,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1167,7 +1147,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1178,7 +1158,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1189,7 +1169,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1200,7 +1180,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1211,7 +1191,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1222,7 +1202,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1233,7 +1213,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1244,7 +1224,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1255,7 +1235,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1266,7 +1246,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1277,7 +1257,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1288,7 +1268,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1299,7 +1279,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>NMIH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1310,7 +1290,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1321,7 +1301,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>NWBI</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1332,7 +1312,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1343,7 +1323,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1354,7 +1334,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1365,7 +1345,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1376,7 +1356,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1387,7 +1367,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>PAYO</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1398,11 +1378,165 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SBCF</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-27
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,11 +444,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>BKR</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>AMBA</t>
@@ -456,30 +452,26 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ACT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LSTR</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANIP</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -493,18 +485,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
@@ -517,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -536,13 +528,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -555,13 +547,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -569,18 +561,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>CALY</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
@@ -588,18 +580,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -607,18 +599,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BUSE</t>
         </is>
       </c>
     </row>
@@ -626,18 +618,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CFR</t>
         </is>
       </c>
     </row>
@@ -645,18 +637,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CENTA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -664,18 +656,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>EXTR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>CGNT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
@@ -683,18 +675,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
@@ -702,18 +694,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
@@ -721,18 +713,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -740,93 +732,113 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NXST</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>OSIS</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>FANG</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PATK</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>FITB</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>FFIV</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
@@ -835,13 +847,13 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>FULT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>FTNT</t>
         </is>
       </c>
     </row>
@@ -850,13 +862,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
@@ -865,13 +877,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -880,13 +892,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
@@ -895,13 +907,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -910,13 +922,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
@@ -925,13 +937,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -940,13 +952,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>ICUI</t>
         </is>
       </c>
     </row>
@@ -955,13 +967,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
@@ -970,13 +982,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>LIVN</t>
         </is>
       </c>
     </row>
@@ -985,13 +997,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>NMIH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
@@ -1000,13 +1012,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -1015,528 +1027,191 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>NUTX</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NWBI</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>QLYS</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>SFNC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>SRZN</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>SYRE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>XNCR</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>HQY</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>HTHT</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>HURN</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>ICUI</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>INDB</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>LFST</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>LIN</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>LOGI</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>MEDP</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>MEOH</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>NDAQ</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>NMIH</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>NSIT</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr"/>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>NWBI</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>NWE</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>OSPN</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr"/>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>OZK</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr"/>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr"/>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>PAGP</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>PAYO</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr"/>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>PNFP</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>PTEN</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>QLYS</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>ROST</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>RPRX</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>SBCF</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>SFNC</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>SIGI</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>SWIM</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>SYRE</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-28
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,7 +444,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ENSG</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>AMBA</t>
@@ -452,13 +456,13 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>ABCL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
@@ -466,18 +470,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ABSI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -485,18 +489,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
@@ -509,13 +513,13 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -523,18 +527,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BLBD</t>
+          <t>BOKF</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>ADPT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
@@ -542,18 +546,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BOKF</t>
+          <t>CALY</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>CFR</t>
         </is>
       </c>
     </row>
@@ -561,18 +565,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CALY</t>
+          <t>CARG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
@@ -580,18 +584,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>CERS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
@@ -599,18 +603,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUSE</t>
+          <t>EBC</t>
         </is>
       </c>
     </row>
@@ -618,18 +622,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>CRML</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -637,18 +641,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
@@ -656,18 +660,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
@@ -675,18 +679,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
@@ -694,18 +698,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>ESTA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>BOW</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>GLBE</t>
         </is>
       </c>
     </row>
@@ -713,18 +717,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>BRKR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -732,18 +736,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -751,18 +755,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
@@ -770,18 +774,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>CGNT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>NMIH</t>
         </is>
       </c>
     </row>
@@ -789,18 +793,18 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>OCFC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
@@ -808,18 +812,18 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>OZK</t>
         </is>
       </c>
     </row>
@@ -827,48 +831,56 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>PATK</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>STOK</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>ESQ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>PNFP</t>
         </is>
       </c>
     </row>
@@ -877,13 +889,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
@@ -892,13 +904,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>SFNC</t>
         </is>
       </c>
     </row>
@@ -907,13 +919,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
@@ -922,13 +934,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>STLN</t>
         </is>
       </c>
     </row>
@@ -937,13 +949,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>TCBK</t>
         </is>
       </c>
     </row>
@@ -952,13 +964,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>TECH</t>
         </is>
       </c>
     </row>
@@ -967,13 +979,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
@@ -982,13 +994,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
@@ -997,221 +1009,484 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>LOGI</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>NRIX</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>NTNX</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>GSAT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>NUTX</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>NWBI</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>PAGP</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>PNFP</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>KYMR</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>REGN</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>SLAB</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SYRE</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>TECH</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NBN</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>NOVT</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NUTX</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NWE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>OSW</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>RDNT</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>RDWR</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TGTX</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-29
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,23 +451,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AMBA</t>
+          <t>AAL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FWONK</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>ATMU</t>
@@ -475,13 +479,13 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>ABCL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AFRM</t>
         </is>
       </c>
     </row>
@@ -489,18 +493,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ABSI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>AMCR</t>
         </is>
       </c>
     </row>
@@ -508,18 +512,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>BLBD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
@@ -527,18 +531,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BOKF</t>
+          <t>CALY</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ADPT</t>
+          <t>ACT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -546,18 +550,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CALY</t>
+          <t>CERS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
@@ -565,18 +569,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ADPT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
@@ -584,18 +588,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CERS</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ADUS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
@@ -603,18 +607,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -622,18 +626,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CRML</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>ALKS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
@@ -641,18 +645,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>DRS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
@@ -660,18 +664,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>ELDN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -679,18 +683,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>ESTA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -698,18 +702,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ESTA</t>
+          <t>EVLV</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
@@ -717,18 +721,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>FER</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BRKR</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>FANG</t>
         </is>
       </c>
     </row>
@@ -736,18 +740,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AXGN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
@@ -755,18 +759,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>BOW</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>FSUN</t>
         </is>
       </c>
     </row>
@@ -774,18 +778,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>INDV</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>BRKR</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
@@ -793,18 +797,18 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>OCFC</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -812,18 +816,18 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>NEXT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CFR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>MDB</t>
         </is>
       </c>
     </row>
@@ -831,18 +835,18 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>NDSN</t>
         </is>
       </c>
     </row>
@@ -850,18 +854,18 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>STOK</t>
+          <t>OCFC</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
@@ -869,108 +873,132 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>PTCT</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>STOK</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TBLA</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>TCBK</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>ESQ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
@@ -979,13 +1007,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>SBCF</t>
         </is>
       </c>
     </row>
@@ -994,13 +1022,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
@@ -1009,62 +1037,82 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>FFBC</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>FITB</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1075,7 +1123,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1086,7 +1134,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>FULT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1097,7 +1145,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KYMR</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1108,7 +1156,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1119,7 +1167,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1130,7 +1178,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1141,7 +1189,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1152,7 +1200,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1163,7 +1211,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1174,7 +1222,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NBN</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1185,7 +1233,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1196,7 +1244,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1207,7 +1255,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>KYMR</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1218,7 +1266,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1229,7 +1277,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NUTX</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1240,7 +1288,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1251,7 +1299,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1262,7 +1310,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1273,7 +1321,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1284,7 +1332,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ORKA</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1295,7 +1343,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>MGRC</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1306,7 +1354,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>NBN</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1317,7 +1365,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1328,7 +1376,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>NMIH</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1339,7 +1387,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>RDNT</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1350,7 +1398,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>RDWR</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1361,7 +1409,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>NTRA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1372,7 +1420,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>OABI</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1383,7 +1431,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>RLAY</t>
+          <t>ORKA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1394,7 +1442,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1405,7 +1453,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1416,7 +1464,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SGMT</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1427,7 +1475,7 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -1438,7 +1486,7 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SYRE</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -1449,7 +1497,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TGTX</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -1460,7 +1508,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>VISN</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -1471,7 +1519,7 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>RDNT</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -1482,11 +1530,253 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>RDWR</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>REPL</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SHC</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr"/>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>TCBK</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>TGTX</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>VCTR</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr"/>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-30
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,11 +444,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ENSG</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>AAL</t>
@@ -462,30 +458,26 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ABSI</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>FWONK</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>BCRX</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
@@ -493,18 +485,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>ADPT</t>
         </is>
       </c>
     </row>
@@ -512,18 +504,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BLBD</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ADUS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -531,18 +523,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CALY</t>
+          <t>BOKF</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
@@ -550,18 +542,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CERS</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -569,18 +561,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ADPT</t>
+          <t>ALKS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
@@ -588,18 +580,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CRSP</t>
+          <t>DRS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AMCR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
@@ -607,18 +599,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>EVLV</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BBT</t>
         </is>
       </c>
     </row>
@@ -626,18 +618,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>FTAI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -645,18 +637,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DRS</t>
+          <t>FWONK</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -664,18 +656,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ELDN</t>
+          <t>INDV</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
@@ -683,18 +675,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ESTA</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>AXGN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
@@ -702,18 +694,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EVLV</t>
+          <t>PODC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>BJRI</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>CFR</t>
         </is>
       </c>
     </row>
@@ -721,18 +713,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FER</t>
+          <t>PTCT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>BTSG</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
@@ -740,18 +732,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>RYAAY</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
@@ -759,18 +751,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>RYTM</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FSUN</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
@@ -778,18 +770,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>INDV</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BRKR</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
@@ -797,18 +789,18 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>STOK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>EBC</t>
         </is>
       </c>
     </row>
@@ -816,18 +808,18 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NEXT</t>
+          <t>SUPN</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>ESQ</t>
         </is>
       </c>
     </row>
@@ -835,18 +827,18 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>SVRA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
@@ -854,66 +846,54 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>OCFC</t>
+          <t>TBLA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>PTCT</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>RYAAY</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>FIBK</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>SOFI</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>DLTR</t>
@@ -922,17 +902,13 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>STOK</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>DORM</t>
@@ -941,64 +917,52 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>SUPN</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>GH</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>TBLA</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>TPG</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -1007,13 +971,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SBCF</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
@@ -1022,13 +986,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>KYMR</t>
         </is>
       </c>
     </row>
@@ -1037,13 +1001,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>MSGK</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1022,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -1067,13 +1031,13 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
@@ -1082,13 +1046,13 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -1097,13 +1061,13 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>GEN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>OZK</t>
         </is>
       </c>
     </row>
@@ -1112,227 +1076,307 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>RDNT</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>RDWR</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SBCF</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>LLYVA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TCBK</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>KYMR</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>ORKA</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TLS</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PFG</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1343,7 +1387,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MGRC</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1354,7 +1398,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>NBN</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1365,7 +1409,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1376,7 +1420,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1387,7 +1431,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>PVLA</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1398,7 +1442,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1409,7 +1453,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1420,7 +1464,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1431,7 +1475,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ORKA</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1442,7 +1486,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1453,7 +1497,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>STGW</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1464,7 +1508,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1475,7 +1519,7 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -1486,7 +1530,7 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>TGTX</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -1497,7 +1541,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -1508,7 +1552,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>UTHR</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -1519,264 +1563,11 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>RDNT</t>
+          <t>VCTR</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>RDWR</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>REGN</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>REPL</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>RGEN</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>RLAY</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>ROIV</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr"/>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr"/>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>SFNC</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr"/>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>SGMT</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr"/>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>SHC</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr"/>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr"/>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>STLD</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr"/>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>SYRE</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr"/>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>TCBK</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr"/>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>TEM</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr"/>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr"/>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>TGTX</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr"/>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr"/>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr"/>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>VCTR</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>VISN</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
MACD scan results 2026-10-31
</commit_message>
<xml_diff>
--- a/results/macd_latest.xlsx
+++ b/results/macd_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -471,7 +471,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ADUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -490,13 +490,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ADPT</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AMCR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -542,18 +542,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ASND</t>
         </is>
       </c>
     </row>
@@ -561,12 +561,12 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CRSP</t>
+          <t>DRS</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>ATEX</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -580,18 +580,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DRS</t>
+          <t>EVLV</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>AXGN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
@@ -599,18 +599,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EVLV</t>
+          <t>FER</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>BTSG</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
@@ -623,13 +623,13 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>BBT</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -661,7 +661,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -680,7 +680,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -694,12 +694,12 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PODC</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BJRI</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -713,18 +713,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PTCT</t>
+          <t>PODC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
@@ -737,13 +737,13 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -775,13 +775,13 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>EBC</t>
         </is>
       </c>
     </row>
@@ -794,13 +794,13 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
@@ -813,13 +813,13 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>FIBK</t>
         </is>
       </c>
     </row>
@@ -827,37 +827,33 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SVRA</t>
+          <t>TBLA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>TBLA</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
@@ -866,13 +862,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>GH</t>
         </is>
       </c>
     </row>
@@ -881,13 +877,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -896,13 +892,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
@@ -911,13 +907,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>FRHC</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -926,13 +922,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
@@ -941,13 +937,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>GEN</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
@@ -956,13 +952,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>LECO</t>
         </is>
       </c>
     </row>
@@ -971,13 +967,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
@@ -986,13 +982,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>KYMR</t>
+          <t>MGRC</t>
         </is>
       </c>
     </row>
@@ -1001,7 +997,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>KYMR</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1016,13 +1012,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
@@ -1031,13 +1027,13 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1042,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>LLYVA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1061,7 +1057,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GEN</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1076,7 +1072,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1091,13 +1087,13 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
@@ -1106,13 +1102,13 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>NNBR</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>RDNT</t>
+          <t>PAYO</t>
         </is>
       </c>
     </row>
@@ -1121,13 +1117,13 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>OABI</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>RDWR</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
@@ -1136,13 +1132,13 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>RLAY</t>
+          <t>RDWR</t>
         </is>
       </c>
     </row>
@@ -1151,13 +1147,13 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>ORKA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SBCF</t>
+          <t>ROIV</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1162,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1181,13 +1177,13 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
@@ -1196,13 +1192,13 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SGMT</t>
+          <t>SFNC</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1207,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LLYVA</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1226,7 +1222,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1241,7 +1237,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1256,13 +1252,13 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>TCBK</t>
+          <t>TEM</t>
         </is>
       </c>
     </row>
@@ -1271,13 +1267,13 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>PVLA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
@@ -1286,13 +1282,13 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>RDNT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
@@ -1301,13 +1297,13 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>VCTR</t>
         </is>
       </c>
     </row>
@@ -1316,13 +1312,13 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ORKA</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>VISN</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1327,13 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>VISN</t>
+          <t>VSXY</t>
         </is>
       </c>
     </row>
@@ -1346,37 +1342,29 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PFG</t>
+          <t>SLAB</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>STGW</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1387,7 +1375,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1398,7 +1386,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1409,7 +1397,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>TENB</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1420,7 +1408,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>TGTX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1431,7 +1419,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PVLA</t>
+          <t>TONT</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1442,7 +1430,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1453,7 +1441,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>WTW</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1464,110 +1452,11 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>XNCR</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>RPRX</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr"/>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>STLD</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>SWIM</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>TGTX</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>VCTR</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>